<commit_message>
Added timeout, server messages popup, active textbar on each reload and improvements in the PMS thing
</commit_message>
<xml_diff>
--- a/Result/Inspection_Log.xlsx
+++ b/Result/Inspection_Log.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -4220,6 +4220,378 @@
         </is>
       </c>
     </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 11:51:05</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>SN1234567</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K61" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L61" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 11:53:32</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>PCB-20261026062332</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K62" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L62" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 15:29:12</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K63" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L63" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 16:00:11</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K64" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L64" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 16:38:48</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K65" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L65" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27 09:05:48</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K66" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L66" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed the payload part and made the id static
</commit_message>
<xml_diff>
--- a/Result/Inspection_Log.xlsx
+++ b/Result/Inspection_Log.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inspection Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Inspection Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -4592,6 +4592,316 @@
         </is>
       </c>
     </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27 11:11:08</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K67" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L67" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27 11:15:34</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K68" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L68" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27 11:17:59</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K69" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L69" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27 11:23:04</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K70" s="5" t="inlineStr">
+        <is>
+          <t>Failed: Wire Case 3 (BR)</t>
+        </is>
+      </c>
+      <c r="L70" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27 11:27:03</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K71" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L71" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added the JIg UID logic, tetsing stage, table name conmfigurable and clear the prev test case after scanning the new device
</commit_message>
<xml_diff>
--- a/Result/Inspection_Log.xlsx
+++ b/Result/Inspection_Log.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -4902,6 +4902,688 @@
         </is>
       </c>
     </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 12:10:41</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L72" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 12:15:37</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K73" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L73" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 12:17:04</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K74" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L74" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 15:19:07</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K75" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L75" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 15:21:36</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K76" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L76" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 15:23:25</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K77" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L77" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 16:45:54</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K78" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L78" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 16:47:27</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K79" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L79" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 16:56:15</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K80" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L80" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 16:56:54</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K81" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L81" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 16:59:42</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K82" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L82" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Made changes of pms connection
</commit_message>
<xml_diff>
--- a/Result/Inspection_Log.xlsx
+++ b/Result/Inspection_Log.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -5584,6 +5584,1122 @@
         </is>
       </c>
     </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:21:52</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K83" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L83" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:29:43</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K84" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L84" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:33:41</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K85" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L85" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:37:12</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J86" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K86" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L86" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:48:19</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K87" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L87" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:48:59</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I88" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J88" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K88" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L88" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:53:56</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I89" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J89" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K89" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L89" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 11:04:21</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I90" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J90" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K90" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L90" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 11:04:32</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I91" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J91" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K91" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L91" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 11:46:32</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H92" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I92" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J92" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K92" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L92" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 11:57:57</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I93" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J93" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K93" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L93" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:15:06</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I94" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J94" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K94" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L94" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:22:04</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I95" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J95" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K95" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L95" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:25:54</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I96" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J96" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K96" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L96" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 14:07:39</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I97" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J97" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K97" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L97" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 15:36:35</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I98" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J98" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K98" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L98" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 16:28:10</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I99" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J99" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K99" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L99" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 09:04:27</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I100" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J100" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K100" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L100" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
removed the unnecessary parameter from report store payload and changed the Production Line to GTI version
</commit_message>
<xml_diff>
--- a/Result/Inspection_Log.xlsx
+++ b/Result/Inspection_Log.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -6700,6 +6700,130 @@
         </is>
       </c>
     </row>
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 13:16:33</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F101" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I101" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J101" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K101" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L101" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 13:22:51</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C102" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F102" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H102" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I102" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J102" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K102" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L102" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update wiring detection and inspection workflow
</commit_message>
<xml_diff>
--- a/Result/Inspection_Log.xlsx
+++ b/Result/Inspection_Log.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Inspection Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inspection Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -496,7 +496,7 @@
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="122" customWidth="1" min="11" max="11"/>
+    <col width="131" customWidth="1" min="11" max="11"/>
     <col width="19" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -6824,6 +6824,1494 @@
         </is>
       </c>
     </row>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 09:58:19</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F103" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H103" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K103" s="5" t="inlineStr">
+        <is>
+          <t>Failed: Origin 1 (BL), Origin 2 (UM Coil), Wire Case 1 (BL), Wire Case 2 (UM), Wire Case 3 (BR)</t>
+        </is>
+      </c>
+      <c r="L103" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 10:14:14</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>TEST1234</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F104" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G104" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H104" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I104" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J104" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K104" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L104" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 10:16:10</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H105" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I105" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J105" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K105" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L105" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 10:31:38</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C106" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F106" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G106" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H106" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I106" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J106" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K106" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L106" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="22" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 10:55:50</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>TEST-FAIL-01</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G107" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H107" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="J107" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K107" s="5" t="inlineStr">
+        <is>
+          <t>Failed: Top View (Wire Pose Model): Red and black wires not detected; Side View (Origin 3 Model): Origin 3 grommet not detected</t>
+        </is>
+      </c>
+      <c r="L107" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="22" customHeight="1">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 10:55:50</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>TEST-PASS-01</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H108" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="J108" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K108" s="5" t="inlineStr">
+        <is>
+          <t>Failed: Top View (Wire Pose Model): Red and black wires not detected; Side View (Origin 3 Model): Origin 3 grommet not detected</t>
+        </is>
+      </c>
+      <c r="L108" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="22" customHeight="1">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 10:56:24</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>TEST-FAIL-01</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K109" s="5" t="inlineStr">
+        <is>
+          <t>Failed: Top View (Wire Pose Model): Red and black wires not detected; Side View (Origin 3 Model): Origin 3 grommet not detected</t>
+        </is>
+      </c>
+      <c r="L109" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 10:56:24</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>TEST-PASS-01</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F110" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G110" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H110" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I110" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J110" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K110" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L110" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 11:23:05</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>TEST_PASS_001</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F111" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G111" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H111" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I111" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J111" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K111" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L111" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="22" customHeight="1">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 11:23:05</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>TEST_FAIL_SIDE_001</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H112" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I112" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J112" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K112" s="5" t="inlineStr">
+        <is>
+          <t>Failed Cases: Origin 3 (Side View)</t>
+        </is>
+      </c>
+      <c r="L112" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="22" customHeight="1">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 11:23:05</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>TEST_FAIL_BOTH_001</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K113" s="5" t="inlineStr">
+        <is>
+          <t>Failed Cases: Case 1 (BL), Case 2 (UM), Case 3 (BR), Origin 3 (Side View)</t>
+        </is>
+      </c>
+      <c r="L113" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="22" customHeight="1">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 11:27:12</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C114" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F114" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G114" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H114" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I114" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J114" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K114" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L114" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="22" customHeight="1">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 11:30:34</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F115" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G115" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H115" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I115" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J115" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K115" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L115" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 11:33:33</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F116" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G116" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H116" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I116" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J116" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K116" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L116" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 11:45:25</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>TEST_UNIT_999</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F117" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G117" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H117" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I117" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J117" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K117" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L117" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="22" customHeight="1">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 12:10:39</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>TEST_PASS_001</t>
+        </is>
+      </c>
+      <c r="C118" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F118" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G118" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H118" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I118" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J118" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K118" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L118" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="22" customHeight="1">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 12:10:39</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>TEST_FAIL_SIDE_001</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G119" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H119" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I119" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J119" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K119" s="5" t="inlineStr">
+        <is>
+          <t>Failed Cases: Origin 3 (Grommet)</t>
+        </is>
+      </c>
+      <c r="L119" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="22" customHeight="1">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 12:10:39</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>TEST_FAIL_TOP_001</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F120" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G120" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H120" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I120" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="J120" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K120" s="5" t="inlineStr">
+        <is>
+          <t>Failed Cases: Origin 1 (BL), Origin 2 (UM), Origin 3 (BR Top), Case 1 (BL), Case 2 (UM), Case 3 (BR)</t>
+        </is>
+      </c>
+      <c r="L120" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="22" customHeight="1">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 12:31:13</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F121" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G121" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H121" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I121" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J121" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K121" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L121" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="22" customHeight="1">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 12:31:57</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H122" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I122" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J122" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K122" s="5" t="inlineStr">
+        <is>
+          <t>Failed Cases: Origin 1 (BL), Case 1 (BL)</t>
+        </is>
+      </c>
+      <c r="L122" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="22" customHeight="1">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 13:29:14</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>TEST_PASS_001</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F123" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G123" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H123" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I123" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J123" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K123" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L123" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="22" customHeight="1">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 13:29:14</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>TEST_FAIL_SIDE_001</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G124" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H124" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I124" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J124" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K124" s="5" t="inlineStr">
+        <is>
+          <t>Failed Cases: Origin 3 (Grommet)</t>
+        </is>
+      </c>
+      <c r="L124" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="22" customHeight="1">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 13:29:14</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>TEST_FAIL_TOP_001</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F125" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="H125" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I125" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="J125" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="K125" s="5" t="inlineStr">
+        <is>
+          <t>Failed Cases: Origin 1 (BL), Origin 2 (UM), Origin 3 (BR Top), Case 1 (BL), Case 2 (UM), Case 3 (BR)</t>
+        </is>
+      </c>
+      <c r="L125" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="22" customHeight="1">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 13:40:09</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F126" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G126" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H126" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I126" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J126" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K126" s="5" t="inlineStr">
+        <is>
+          <t>Failed Cases: Origin 1 (BL)</t>
+        </is>
+      </c>
+      <c r="L126" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Change the report store from various parameter to viInspection and remarks
</commit_message>
<xml_diff>
--- a/Result/Inspection_Log.xlsx
+++ b/Result/Inspection_Log.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inspection Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Inspection Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -8312,6 +8312,192 @@
         </is>
       </c>
     </row>
+    <row r="127" ht="22" customHeight="1">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 14:20:21</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E127" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F127" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G127" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H127" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I127" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J127" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K127" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L127" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="22" customHeight="1">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 14:41:13</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F128" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G128" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H128" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I128" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J128" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K128" s="5" t="inlineStr">
+        <is>
+          <t>All checks passed</t>
+        </is>
+      </c>
+      <c r="L128" s="5" t="inlineStr">
+        <is>
+          <t>Result/Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="22" customHeight="1">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 14:42:50</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>001260101010112105100002607001973</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E129" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F129" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G129" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H129" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I129" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J129" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K129" s="5" t="inlineStr">
+        <is>
+          <t>Failed Cases: Origin 1 (BL)</t>
+        </is>
+      </c>
+      <c r="L129" s="5" t="inlineStr">
+        <is>
+          <t>Result/Fail</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>